<commit_message>
Finance v3: founder questions with numbers, bills tracker, 6-month P&L (20/50/100 hostels), morning checklist
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0191SJ1qAdm8xL7m212nsCqQ
</commit_message>
<xml_diff>
--- a/docs/finance/hostelzy-money.xlsx
+++ b/docs/finance/hostelzy-money.xlsx
@@ -8,12 +8,14 @@
   </bookViews>
   <sheets>
     <sheet name="How to use" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Budget" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Money in" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Money out" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Rewards" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Partners" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Summary" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Bills" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="P&amp;L" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Budget" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Money in" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Money out" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Rewards" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Partners" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Summary" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -22,7 +24,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
+  <numFmts count="2">
+    <numFmt numFmtId="164" formatCode="₹#,##0"/>
+    <numFmt numFmtId="165" formatCode="₹#,##0;[Red]-₹#,##0"/>
+  </numFmts>
   <fonts count="3">
     <font>
       <name val="Calibri"/>
@@ -39,7 +44,7 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -49,6 +54,16 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00EC3013"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EEEEEE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF3B0"/>
       </patternFill>
     </fill>
   </fills>
@@ -64,12 +79,18 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="9" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -435,7 +456,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B8"/>
+  <dimension ref="A1:B9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -524,12 +545,2108 @@
         </is>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Bills tab: every account the app needs, cost and due date. P&amp;L tab: 6-month P&amp;L at 20/50/100 hostels; edit yellow cells.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G13"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="28" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="40" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>Account</t>
+        </is>
+      </c>
+      <c r="B1" s="3" t="inlineStr">
+        <is>
+          <t>Plan</t>
+        </is>
+      </c>
+      <c r="C1" s="3" t="inlineStr">
+        <is>
+          <t>₹ per month</t>
+        </is>
+      </c>
+      <c r="D1" s="3" t="inlineStr">
+        <is>
+          <t>₹ one time / yearly</t>
+        </is>
+      </c>
+      <c r="E1" s="3" t="inlineStr">
+        <is>
+          <t>Due</t>
+        </is>
+      </c>
+      <c r="F1" s="3" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="G1" s="3" t="inlineStr">
+        <is>
+          <t>Unblocks</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Google Play Console</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>One time $25</t>
+        </is>
+      </c>
+      <c r="C2" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D2" s="4" t="n">
+        <v>2900</v>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Week of 6 Oct 2026</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Not paid</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Play upload + 14-day closed test</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Supabase live (Mumbai)</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Free → Pro $25/mo</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="n">
+        <v>2900</v>
+      </c>
+      <c r="D3" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>1 Nov 2026</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Free, running</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Backups, no pausing, real owners' data</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Supabase staging</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D4" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>When Build needs it</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Not made</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Test SQL before the live run</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Firebase Spark</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D5" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Running</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Google sign-in, push, crashes</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Firebase Blaze (SMS OTP)</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Pay per SMS, ₹1,000 alert</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="n">
+        <v>1000</v>
+      </c>
+      <c r="D6" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Nov 2026 (card)</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Card failed once</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Verified phones</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Google Maps SDK</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Pay as you go, ₹500 alert</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D7" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Before Play launch</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Not set up</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Real map at launch</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>MapTiler (fallback only)</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Flex ~$25/mo</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D8" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Only if Google fails</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Map without a Google card</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Domain hostelzy.in</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Yearly</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D9" s="4" t="n">
+        <v>800</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Oct 2026</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Not bought</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Own web address</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>GitHub Pro</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>$4/mo when repo private</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="n">
+        <v>460</v>
+      </c>
+      <c r="D10" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>When repo goes private</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>Pages + build minutes on private repo</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Claude / AI tokens</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Your plan</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="n">
+        <v>10000</v>
+      </c>
+      <c r="D11" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Monthly</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Running</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>Building the app</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>WhatsApp Business app</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="C12" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D12" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>Owner chats</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr"/>
+      <c r="C13" s="5">
+        <f>SUM(C2:C12)</f>
+        <v/>
+      </c>
+      <c r="D13" s="5">
+        <f>SUM(D2:D12)</f>
+        <v/>
+      </c>
+      <c r="E13" s="2" t="inlineStr"/>
+      <c r="F13" s="2" t="inlineStr"/>
+      <c r="G13" s="2" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:M64"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="44" customWidth="1" min="1" max="1"/>
+    <col width="13" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="13" customWidth="1" min="8" max="8"/>
+    <col width="13" customWidth="1" min="9" max="9"/>
+    <col width="13" customWidth="1" min="10" max="10"/>
+    <col width="13" customWidth="1" min="11" max="11"/>
+    <col width="13" customWidth="1" min="12" max="12"/>
+    <col width="13" customWidth="1" min="13" max="13"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>Assumptions (edit the yellow cells)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Average price per paying hostel (₹)</t>
+        </is>
+      </c>
+      <c r="B2" s="6" t="n">
+        <v>750</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Trial converts to paid</t>
+        </is>
+      </c>
+      <c r="B3" s="7" t="n">
+        <v>0.7</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Commission per new paying owner (₹)</t>
+        </is>
+      </c>
+      <c r="B4" s="6" t="n">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Print per new hostel (₹)</t>
+        </is>
+      </c>
+      <c r="B5" s="6" t="n">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Rewards per paying hostel (₹, from month 3)</t>
+        </is>
+      </c>
+      <c r="B6" s="6" t="n">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Rewards cap (₹)</t>
+        </is>
+      </c>
+      <c r="B7" s="6" t="n">
+        <v>5000</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>AI tokens (₹/month)</t>
+        </is>
+      </c>
+      <c r="B8" s="6" t="n">
+        <v>10000</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Tech month 1 (₹)</t>
+        </is>
+      </c>
+      <c r="B9" s="6" t="n">
+        <v>4260</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Tech base from month 2 (₹, + SMS)</t>
+        </is>
+      </c>
+      <c r="B10" s="6" t="n">
+        <v>3360</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>Scenario: 20 hostels by March</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>SMS ₹/mo</t>
+        </is>
+      </c>
+      <c r="I12" s="6" t="n">
+        <v>500</v>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>Hold pay ₹/mo</t>
+        </is>
+      </c>
+      <c r="K12" s="6" t="n">
+        <v>1000</v>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>Ads ₹/mo</t>
+        </is>
+      </c>
+      <c r="M12" s="6" t="n">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>Line</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>Oct 2026</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>Nov 2026</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>Dec 2026</t>
+        </is>
+      </c>
+      <c r="E13" s="3" t="inlineStr">
+        <is>
+          <t>Jan 2027</t>
+        </is>
+      </c>
+      <c r="F13" s="3" t="inlineStr">
+        <is>
+          <t>Feb 2027</t>
+        </is>
+      </c>
+      <c r="G13" s="3" t="inlineStr">
+        <is>
+          <t>Mar 2027</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Hostels live</t>
+        </is>
+      </c>
+      <c r="B14" s="6" t="n">
+        <v>15</v>
+      </c>
+      <c r="C14" s="6" t="n">
+        <v>20</v>
+      </c>
+      <c r="D14" s="6" t="n">
+        <v>20</v>
+      </c>
+      <c r="E14" s="6" t="n">
+        <v>20</v>
+      </c>
+      <c r="F14" s="6" t="n">
+        <v>20</v>
+      </c>
+      <c r="G14" s="6" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Paying hostels</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>0</v>
+      </c>
+      <c r="C15">
+        <f>ROUND($B$3*B14,0)</f>
+        <v/>
+      </c>
+      <c r="D15">
+        <f>ROUND($B$3*C14,0)</f>
+        <v/>
+      </c>
+      <c r="E15">
+        <f>ROUND($B$3*D14,0)</f>
+        <v/>
+      </c>
+      <c r="F15">
+        <f>ROUND($B$3*E14,0)</f>
+        <v/>
+      </c>
+      <c r="G15">
+        <f>ROUND($B$3*F14,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>Revenue</t>
+        </is>
+      </c>
+      <c r="B16" s="8">
+        <f>$B$2*B15</f>
+        <v/>
+      </c>
+      <c r="C16" s="8">
+        <f>$B$2*C15</f>
+        <v/>
+      </c>
+      <c r="D16" s="8">
+        <f>$B$2*D15</f>
+        <v/>
+      </c>
+      <c r="E16" s="8">
+        <f>$B$2*E15</f>
+        <v/>
+      </c>
+      <c r="F16" s="8">
+        <f>$B$2*F15</f>
+        <v/>
+      </c>
+      <c r="G16" s="8">
+        <f>$B$2*G15</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Tech</t>
+        </is>
+      </c>
+      <c r="B17" s="8">
+        <f>$B$9</f>
+        <v/>
+      </c>
+      <c r="C17" s="8">
+        <f>$B$10+$I$12</f>
+        <v/>
+      </c>
+      <c r="D17" s="8">
+        <f>$B$10+$I$12</f>
+        <v/>
+      </c>
+      <c r="E17" s="8">
+        <f>$B$10+$I$12</f>
+        <v/>
+      </c>
+      <c r="F17" s="8">
+        <f>$B$10+$I$12</f>
+        <v/>
+      </c>
+      <c r="G17" s="8">
+        <f>$B$10+$I$12</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>AI tokens</t>
+        </is>
+      </c>
+      <c r="B18" s="8">
+        <f>$B$8</f>
+        <v/>
+      </c>
+      <c r="C18" s="8">
+        <f>$B$8</f>
+        <v/>
+      </c>
+      <c r="D18" s="8">
+        <f>$B$8</f>
+        <v/>
+      </c>
+      <c r="E18" s="8">
+        <f>$B$8</f>
+        <v/>
+      </c>
+      <c r="F18" s="8">
+        <f>$B$8</f>
+        <v/>
+      </c>
+      <c r="G18" s="8">
+        <f>$B$8</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Commission</t>
+        </is>
+      </c>
+      <c r="B19" s="8">
+        <f>0</f>
+        <v/>
+      </c>
+      <c r="C19" s="8">
+        <f>$B$4*MAX(0,C15-B15)+$K$12</f>
+        <v/>
+      </c>
+      <c r="D19" s="8">
+        <f>$B$4*MAX(0,D15-C15)+$K$12</f>
+        <v/>
+      </c>
+      <c r="E19" s="8">
+        <f>$B$4*MAX(0,E15-D15)+$K$12</f>
+        <v/>
+      </c>
+      <c r="F19" s="8">
+        <f>$B$4*MAX(0,F15-E15)+$K$12</f>
+        <v/>
+      </c>
+      <c r="G19" s="8">
+        <f>$B$4*MAX(0,G15-F15)+$K$12</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Print</t>
+        </is>
+      </c>
+      <c r="B20" s="8">
+        <f>$B$5*B14</f>
+        <v/>
+      </c>
+      <c r="C20" s="8">
+        <f>$B$5*MAX(0,C14-B14)</f>
+        <v/>
+      </c>
+      <c r="D20" s="8">
+        <f>$B$5*MAX(0,D14-C14)</f>
+        <v/>
+      </c>
+      <c r="E20" s="8">
+        <f>$B$5*MAX(0,E14-D14)</f>
+        <v/>
+      </c>
+      <c r="F20" s="8">
+        <f>$B$5*MAX(0,F14-E14)</f>
+        <v/>
+      </c>
+      <c r="G20" s="8">
+        <f>$B$5*MAX(0,G14-F14)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Travel</t>
+        </is>
+      </c>
+      <c r="B21" s="8">
+        <f>3000</f>
+        <v/>
+      </c>
+      <c r="C21" s="8">
+        <f>IF(C14&gt;B14,3000,1000)</f>
+        <v/>
+      </c>
+      <c r="D21" s="8">
+        <f>IF(D14&gt;C14,3000,1000)</f>
+        <v/>
+      </c>
+      <c r="E21" s="8">
+        <f>IF(E14&gt;D14,3000,1000)</f>
+        <v/>
+      </c>
+      <c r="F21" s="8">
+        <f>IF(F14&gt;E14,3000,1000)</f>
+        <v/>
+      </c>
+      <c r="G21" s="8">
+        <f>IF(G14&gt;F14,3000,1000)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Ads</t>
+        </is>
+      </c>
+      <c r="B22" s="8">
+        <f>0</f>
+        <v/>
+      </c>
+      <c r="C22" s="8">
+        <f>$M$12</f>
+        <v/>
+      </c>
+      <c r="D22" s="8">
+        <f>$M$12</f>
+        <v/>
+      </c>
+      <c r="E22" s="8">
+        <f>$M$12</f>
+        <v/>
+      </c>
+      <c r="F22" s="8">
+        <f>$M$12</f>
+        <v/>
+      </c>
+      <c r="G22" s="8">
+        <f>$M$12</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Rewards</t>
+        </is>
+      </c>
+      <c r="B23" s="8">
+        <f>0</f>
+        <v/>
+      </c>
+      <c r="C23" s="8">
+        <f>0</f>
+        <v/>
+      </c>
+      <c r="D23" s="8">
+        <f>MIN($B$7,$B$6*D15)</f>
+        <v/>
+      </c>
+      <c r="E23" s="8">
+        <f>MIN($B$7,$B$6*E15)</f>
+        <v/>
+      </c>
+      <c r="F23" s="8">
+        <f>MIN($B$7,$B$6*F15)</f>
+        <v/>
+      </c>
+      <c r="G23" s="8">
+        <f>MIN($B$7,$B$6*G15)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>Costs</t>
+        </is>
+      </c>
+      <c r="B24" s="8">
+        <f>SUM(B17:B23)</f>
+        <v/>
+      </c>
+      <c r="C24" s="8">
+        <f>SUM(C17:C23)</f>
+        <v/>
+      </c>
+      <c r="D24" s="8">
+        <f>SUM(D17:D23)</f>
+        <v/>
+      </c>
+      <c r="E24" s="8">
+        <f>SUM(E17:E23)</f>
+        <v/>
+      </c>
+      <c r="F24" s="8">
+        <f>SUM(F17:F23)</f>
+        <v/>
+      </c>
+      <c r="G24" s="8">
+        <f>SUM(G17:G23)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>Profit / loss</t>
+        </is>
+      </c>
+      <c r="B25" s="8">
+        <f>B16-B24</f>
+        <v/>
+      </c>
+      <c r="C25" s="8">
+        <f>C16-C24</f>
+        <v/>
+      </c>
+      <c r="D25" s="8">
+        <f>D16-D24</f>
+        <v/>
+      </c>
+      <c r="E25" s="8">
+        <f>E16-E24</f>
+        <v/>
+      </c>
+      <c r="F25" s="8">
+        <f>F16-F24</f>
+        <v/>
+      </c>
+      <c r="G25" s="8">
+        <f>G16-G24</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>P/L without AI tokens</t>
+        </is>
+      </c>
+      <c r="B26" s="8">
+        <f>B25+B18</f>
+        <v/>
+      </c>
+      <c r="C26" s="8">
+        <f>C25+C18</f>
+        <v/>
+      </c>
+      <c r="D26" s="8">
+        <f>D25+D18</f>
+        <v/>
+      </c>
+      <c r="E26" s="8">
+        <f>E25+E18</f>
+        <v/>
+      </c>
+      <c r="F26" s="8">
+        <f>F25+F18</f>
+        <v/>
+      </c>
+      <c r="G26" s="8">
+        <f>G25+G18</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Cumulative P/L</t>
+        </is>
+      </c>
+      <c r="B27" s="8">
+        <f>B25</f>
+        <v/>
+      </c>
+      <c r="C27" s="8">
+        <f>B27+C25</f>
+        <v/>
+      </c>
+      <c r="D27" s="8">
+        <f>C27+D25</f>
+        <v/>
+      </c>
+      <c r="E27" s="8">
+        <f>D27+E25</f>
+        <v/>
+      </c>
+      <c r="F27" s="8">
+        <f>E27+F25</f>
+        <v/>
+      </c>
+      <c r="G27" s="8">
+        <f>F27+G25</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>Break-even month</t>
+        </is>
+      </c>
+      <c r="B28">
+        <f>IFERROR(INDEX($B$13:$G$13,MATCH(TRUE,INDEX($B$25:$G$25&gt;=0,0),0)),"Not in 6 months")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>Scenario: 50 hostels by March</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>SMS ₹/mo</t>
+        </is>
+      </c>
+      <c r="I30" s="6" t="n">
+        <v>1000</v>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>Hold pay ₹/mo</t>
+        </is>
+      </c>
+      <c r="K30" s="6" t="n">
+        <v>2000</v>
+      </c>
+      <c r="L30" t="inlineStr">
+        <is>
+          <t>Ads ₹/mo</t>
+        </is>
+      </c>
+      <c r="M30" s="6" t="n">
+        <v>2000</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>Line</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="inlineStr">
+        <is>
+          <t>Oct 2026</t>
+        </is>
+      </c>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>Nov 2026</t>
+        </is>
+      </c>
+      <c r="D31" s="3" t="inlineStr">
+        <is>
+          <t>Dec 2026</t>
+        </is>
+      </c>
+      <c r="E31" s="3" t="inlineStr">
+        <is>
+          <t>Jan 2027</t>
+        </is>
+      </c>
+      <c r="F31" s="3" t="inlineStr">
+        <is>
+          <t>Feb 2027</t>
+        </is>
+      </c>
+      <c r="G31" s="3" t="inlineStr">
+        <is>
+          <t>Mar 2027</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Hostels live</t>
+        </is>
+      </c>
+      <c r="B32" s="6" t="n">
+        <v>20</v>
+      </c>
+      <c r="C32" s="6" t="n">
+        <v>30</v>
+      </c>
+      <c r="D32" s="6" t="n">
+        <v>40</v>
+      </c>
+      <c r="E32" s="6" t="n">
+        <v>50</v>
+      </c>
+      <c r="F32" s="6" t="n">
+        <v>50</v>
+      </c>
+      <c r="G32" s="6" t="n">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Paying hostels</t>
+        </is>
+      </c>
+      <c r="B33" t="n">
+        <v>0</v>
+      </c>
+      <c r="C33">
+        <f>ROUND($B$3*B32,0)</f>
+        <v/>
+      </c>
+      <c r="D33">
+        <f>ROUND($B$3*C32,0)</f>
+        <v/>
+      </c>
+      <c r="E33">
+        <f>ROUND($B$3*D32,0)</f>
+        <v/>
+      </c>
+      <c r="F33">
+        <f>ROUND($B$3*E32,0)</f>
+        <v/>
+      </c>
+      <c r="G33">
+        <f>ROUND($B$3*F32,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>Revenue</t>
+        </is>
+      </c>
+      <c r="B34" s="8">
+        <f>$B$2*B33</f>
+        <v/>
+      </c>
+      <c r="C34" s="8">
+        <f>$B$2*C33</f>
+        <v/>
+      </c>
+      <c r="D34" s="8">
+        <f>$B$2*D33</f>
+        <v/>
+      </c>
+      <c r="E34" s="8">
+        <f>$B$2*E33</f>
+        <v/>
+      </c>
+      <c r="F34" s="8">
+        <f>$B$2*F33</f>
+        <v/>
+      </c>
+      <c r="G34" s="8">
+        <f>$B$2*G33</f>
+        <v/>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Tech</t>
+        </is>
+      </c>
+      <c r="B35" s="8">
+        <f>$B$9</f>
+        <v/>
+      </c>
+      <c r="C35" s="8">
+        <f>$B$10+$I$30</f>
+        <v/>
+      </c>
+      <c r="D35" s="8">
+        <f>$B$10+$I$30</f>
+        <v/>
+      </c>
+      <c r="E35" s="8">
+        <f>$B$10+$I$30</f>
+        <v/>
+      </c>
+      <c r="F35" s="8">
+        <f>$B$10+$I$30</f>
+        <v/>
+      </c>
+      <c r="G35" s="8">
+        <f>$B$10+$I$30</f>
+        <v/>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>AI tokens</t>
+        </is>
+      </c>
+      <c r="B36" s="8">
+        <f>$B$8</f>
+        <v/>
+      </c>
+      <c r="C36" s="8">
+        <f>$B$8</f>
+        <v/>
+      </c>
+      <c r="D36" s="8">
+        <f>$B$8</f>
+        <v/>
+      </c>
+      <c r="E36" s="8">
+        <f>$B$8</f>
+        <v/>
+      </c>
+      <c r="F36" s="8">
+        <f>$B$8</f>
+        <v/>
+      </c>
+      <c r="G36" s="8">
+        <f>$B$8</f>
+        <v/>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Commission</t>
+        </is>
+      </c>
+      <c r="B37" s="8">
+        <f>0</f>
+        <v/>
+      </c>
+      <c r="C37" s="8">
+        <f>$B$4*MAX(0,C33-B33)+$K$30</f>
+        <v/>
+      </c>
+      <c r="D37" s="8">
+        <f>$B$4*MAX(0,D33-C33)+$K$30</f>
+        <v/>
+      </c>
+      <c r="E37" s="8">
+        <f>$B$4*MAX(0,E33-D33)+$K$30</f>
+        <v/>
+      </c>
+      <c r="F37" s="8">
+        <f>$B$4*MAX(0,F33-E33)+$K$30</f>
+        <v/>
+      </c>
+      <c r="G37" s="8">
+        <f>$B$4*MAX(0,G33-F33)+$K$30</f>
+        <v/>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Print</t>
+        </is>
+      </c>
+      <c r="B38" s="8">
+        <f>$B$5*B32</f>
+        <v/>
+      </c>
+      <c r="C38" s="8">
+        <f>$B$5*MAX(0,C32-B32)</f>
+        <v/>
+      </c>
+      <c r="D38" s="8">
+        <f>$B$5*MAX(0,D32-C32)</f>
+        <v/>
+      </c>
+      <c r="E38" s="8">
+        <f>$B$5*MAX(0,E32-D32)</f>
+        <v/>
+      </c>
+      <c r="F38" s="8">
+        <f>$B$5*MAX(0,F32-E32)</f>
+        <v/>
+      </c>
+      <c r="G38" s="8">
+        <f>$B$5*MAX(0,G32-F32)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Travel</t>
+        </is>
+      </c>
+      <c r="B39" s="8">
+        <f>3000</f>
+        <v/>
+      </c>
+      <c r="C39" s="8">
+        <f>IF(C32&gt;B32,3000,1000)</f>
+        <v/>
+      </c>
+      <c r="D39" s="8">
+        <f>IF(D32&gt;C32,3000,1000)</f>
+        <v/>
+      </c>
+      <c r="E39" s="8">
+        <f>IF(E32&gt;D32,3000,1000)</f>
+        <v/>
+      </c>
+      <c r="F39" s="8">
+        <f>IF(F32&gt;E32,3000,1000)</f>
+        <v/>
+      </c>
+      <c r="G39" s="8">
+        <f>IF(G32&gt;F32,3000,1000)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Ads</t>
+        </is>
+      </c>
+      <c r="B40" s="8">
+        <f>0</f>
+        <v/>
+      </c>
+      <c r="C40" s="8">
+        <f>$M$30</f>
+        <v/>
+      </c>
+      <c r="D40" s="8">
+        <f>$M$30</f>
+        <v/>
+      </c>
+      <c r="E40" s="8">
+        <f>$M$30</f>
+        <v/>
+      </c>
+      <c r="F40" s="8">
+        <f>$M$30</f>
+        <v/>
+      </c>
+      <c r="G40" s="8">
+        <f>$M$30</f>
+        <v/>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Rewards</t>
+        </is>
+      </c>
+      <c r="B41" s="8">
+        <f>0</f>
+        <v/>
+      </c>
+      <c r="C41" s="8">
+        <f>0</f>
+        <v/>
+      </c>
+      <c r="D41" s="8">
+        <f>MIN($B$7,$B$6*D33)</f>
+        <v/>
+      </c>
+      <c r="E41" s="8">
+        <f>MIN($B$7,$B$6*E33)</f>
+        <v/>
+      </c>
+      <c r="F41" s="8">
+        <f>MIN($B$7,$B$6*F33)</f>
+        <v/>
+      </c>
+      <c r="G41" s="8">
+        <f>MIN($B$7,$B$6*G33)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="inlineStr">
+        <is>
+          <t>Costs</t>
+        </is>
+      </c>
+      <c r="B42" s="8">
+        <f>SUM(B35:B41)</f>
+        <v/>
+      </c>
+      <c r="C42" s="8">
+        <f>SUM(C35:C41)</f>
+        <v/>
+      </c>
+      <c r="D42" s="8">
+        <f>SUM(D35:D41)</f>
+        <v/>
+      </c>
+      <c r="E42" s="8">
+        <f>SUM(E35:E41)</f>
+        <v/>
+      </c>
+      <c r="F42" s="8">
+        <f>SUM(F35:F41)</f>
+        <v/>
+      </c>
+      <c r="G42" s="8">
+        <f>SUM(G35:G41)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="2" t="inlineStr">
+        <is>
+          <t>Profit / loss</t>
+        </is>
+      </c>
+      <c r="B43" s="8">
+        <f>B34-B42</f>
+        <v/>
+      </c>
+      <c r="C43" s="8">
+        <f>C34-C42</f>
+        <v/>
+      </c>
+      <c r="D43" s="8">
+        <f>D34-D42</f>
+        <v/>
+      </c>
+      <c r="E43" s="8">
+        <f>E34-E42</f>
+        <v/>
+      </c>
+      <c r="F43" s="8">
+        <f>F34-F42</f>
+        <v/>
+      </c>
+      <c r="G43" s="8">
+        <f>G34-G42</f>
+        <v/>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>P/L without AI tokens</t>
+        </is>
+      </c>
+      <c r="B44" s="8">
+        <f>B43+B36</f>
+        <v/>
+      </c>
+      <c r="C44" s="8">
+        <f>C43+C36</f>
+        <v/>
+      </c>
+      <c r="D44" s="8">
+        <f>D43+D36</f>
+        <v/>
+      </c>
+      <c r="E44" s="8">
+        <f>E43+E36</f>
+        <v/>
+      </c>
+      <c r="F44" s="8">
+        <f>F43+F36</f>
+        <v/>
+      </c>
+      <c r="G44" s="8">
+        <f>G43+G36</f>
+        <v/>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Cumulative P/L</t>
+        </is>
+      </c>
+      <c r="B45" s="8">
+        <f>B43</f>
+        <v/>
+      </c>
+      <c r="C45" s="8">
+        <f>B45+C43</f>
+        <v/>
+      </c>
+      <c r="D45" s="8">
+        <f>C45+D43</f>
+        <v/>
+      </c>
+      <c r="E45" s="8">
+        <f>D45+E43</f>
+        <v/>
+      </c>
+      <c r="F45" s="8">
+        <f>E45+F43</f>
+        <v/>
+      </c>
+      <c r="G45" s="8">
+        <f>F45+G43</f>
+        <v/>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="inlineStr">
+        <is>
+          <t>Break-even month</t>
+        </is>
+      </c>
+      <c r="B46">
+        <f>IFERROR(INDEX($B$31:$G$31,MATCH(TRUE,INDEX($B$43:$G$43&gt;=0,0),0)),"Not in 6 months")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="2" t="inlineStr">
+        <is>
+          <t>Scenario: 100 hostels by March</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>SMS ₹/mo</t>
+        </is>
+      </c>
+      <c r="I48" s="6" t="n">
+        <v>2000</v>
+      </c>
+      <c r="J48" t="inlineStr">
+        <is>
+          <t>Hold pay ₹/mo</t>
+        </is>
+      </c>
+      <c r="K48" s="6" t="n">
+        <v>4000</v>
+      </c>
+      <c r="L48" t="inlineStr">
+        <is>
+          <t>Ads ₹/mo</t>
+        </is>
+      </c>
+      <c r="M48" s="6" t="n">
+        <v>2000</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="2" t="inlineStr">
+        <is>
+          <t>Line</t>
+        </is>
+      </c>
+      <c r="B49" s="3" t="inlineStr">
+        <is>
+          <t>Oct 2026</t>
+        </is>
+      </c>
+      <c r="C49" s="3" t="inlineStr">
+        <is>
+          <t>Nov 2026</t>
+        </is>
+      </c>
+      <c r="D49" s="3" t="inlineStr">
+        <is>
+          <t>Dec 2026</t>
+        </is>
+      </c>
+      <c r="E49" s="3" t="inlineStr">
+        <is>
+          <t>Jan 2027</t>
+        </is>
+      </c>
+      <c r="F49" s="3" t="inlineStr">
+        <is>
+          <t>Feb 2027</t>
+        </is>
+      </c>
+      <c r="G49" s="3" t="inlineStr">
+        <is>
+          <t>Mar 2027</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>Hostels live</t>
+        </is>
+      </c>
+      <c r="B50" s="6" t="n">
+        <v>20</v>
+      </c>
+      <c r="C50" s="6" t="n">
+        <v>35</v>
+      </c>
+      <c r="D50" s="6" t="n">
+        <v>50</v>
+      </c>
+      <c r="E50" s="6" t="n">
+        <v>70</v>
+      </c>
+      <c r="F50" s="6" t="n">
+        <v>85</v>
+      </c>
+      <c r="G50" s="6" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>Paying hostels</t>
+        </is>
+      </c>
+      <c r="B51" t="n">
+        <v>0</v>
+      </c>
+      <c r="C51">
+        <f>ROUND($B$3*B50,0)</f>
+        <v/>
+      </c>
+      <c r="D51">
+        <f>ROUND($B$3*C50,0)</f>
+        <v/>
+      </c>
+      <c r="E51">
+        <f>ROUND($B$3*D50,0)</f>
+        <v/>
+      </c>
+      <c r="F51">
+        <f>ROUND($B$3*E50,0)</f>
+        <v/>
+      </c>
+      <c r="G51">
+        <f>ROUND($B$3*F50,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="2" t="inlineStr">
+        <is>
+          <t>Revenue</t>
+        </is>
+      </c>
+      <c r="B52" s="8">
+        <f>$B$2*B51</f>
+        <v/>
+      </c>
+      <c r="C52" s="8">
+        <f>$B$2*C51</f>
+        <v/>
+      </c>
+      <c r="D52" s="8">
+        <f>$B$2*D51</f>
+        <v/>
+      </c>
+      <c r="E52" s="8">
+        <f>$B$2*E51</f>
+        <v/>
+      </c>
+      <c r="F52" s="8">
+        <f>$B$2*F51</f>
+        <v/>
+      </c>
+      <c r="G52" s="8">
+        <f>$B$2*G51</f>
+        <v/>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>Tech</t>
+        </is>
+      </c>
+      <c r="B53" s="8">
+        <f>$B$9</f>
+        <v/>
+      </c>
+      <c r="C53" s="8">
+        <f>$B$10+$I$48</f>
+        <v/>
+      </c>
+      <c r="D53" s="8">
+        <f>$B$10+$I$48</f>
+        <v/>
+      </c>
+      <c r="E53" s="8">
+        <f>$B$10+$I$48</f>
+        <v/>
+      </c>
+      <c r="F53" s="8">
+        <f>$B$10+$I$48</f>
+        <v/>
+      </c>
+      <c r="G53" s="8">
+        <f>$B$10+$I$48</f>
+        <v/>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>AI tokens</t>
+        </is>
+      </c>
+      <c r="B54" s="8">
+        <f>$B$8</f>
+        <v/>
+      </c>
+      <c r="C54" s="8">
+        <f>$B$8</f>
+        <v/>
+      </c>
+      <c r="D54" s="8">
+        <f>$B$8</f>
+        <v/>
+      </c>
+      <c r="E54" s="8">
+        <f>$B$8</f>
+        <v/>
+      </c>
+      <c r="F54" s="8">
+        <f>$B$8</f>
+        <v/>
+      </c>
+      <c r="G54" s="8">
+        <f>$B$8</f>
+        <v/>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>Commission</t>
+        </is>
+      </c>
+      <c r="B55" s="8">
+        <f>0</f>
+        <v/>
+      </c>
+      <c r="C55" s="8">
+        <f>$B$4*MAX(0,C51-B51)+$K$48</f>
+        <v/>
+      </c>
+      <c r="D55" s="8">
+        <f>$B$4*MAX(0,D51-C51)+$K$48</f>
+        <v/>
+      </c>
+      <c r="E55" s="8">
+        <f>$B$4*MAX(0,E51-D51)+$K$48</f>
+        <v/>
+      </c>
+      <c r="F55" s="8">
+        <f>$B$4*MAX(0,F51-E51)+$K$48</f>
+        <v/>
+      </c>
+      <c r="G55" s="8">
+        <f>$B$4*MAX(0,G51-F51)+$K$48</f>
+        <v/>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>Print</t>
+        </is>
+      </c>
+      <c r="B56" s="8">
+        <f>$B$5*B50</f>
+        <v/>
+      </c>
+      <c r="C56" s="8">
+        <f>$B$5*MAX(0,C50-B50)</f>
+        <v/>
+      </c>
+      <c r="D56" s="8">
+        <f>$B$5*MAX(0,D50-C50)</f>
+        <v/>
+      </c>
+      <c r="E56" s="8">
+        <f>$B$5*MAX(0,E50-D50)</f>
+        <v/>
+      </c>
+      <c r="F56" s="8">
+        <f>$B$5*MAX(0,F50-E50)</f>
+        <v/>
+      </c>
+      <c r="G56" s="8">
+        <f>$B$5*MAX(0,G50-F50)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>Travel</t>
+        </is>
+      </c>
+      <c r="B57" s="8">
+        <f>3000</f>
+        <v/>
+      </c>
+      <c r="C57" s="8">
+        <f>IF(C50&gt;B50,3000,1000)</f>
+        <v/>
+      </c>
+      <c r="D57" s="8">
+        <f>IF(D50&gt;C50,3000,1000)</f>
+        <v/>
+      </c>
+      <c r="E57" s="8">
+        <f>IF(E50&gt;D50,3000,1000)</f>
+        <v/>
+      </c>
+      <c r="F57" s="8">
+        <f>IF(F50&gt;E50,3000,1000)</f>
+        <v/>
+      </c>
+      <c r="G57" s="8">
+        <f>IF(G50&gt;F50,3000,1000)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>Ads</t>
+        </is>
+      </c>
+      <c r="B58" s="8">
+        <f>0</f>
+        <v/>
+      </c>
+      <c r="C58" s="8">
+        <f>$M$48</f>
+        <v/>
+      </c>
+      <c r="D58" s="8">
+        <f>$M$48</f>
+        <v/>
+      </c>
+      <c r="E58" s="8">
+        <f>$M$48</f>
+        <v/>
+      </c>
+      <c r="F58" s="8">
+        <f>$M$48</f>
+        <v/>
+      </c>
+      <c r="G58" s="8">
+        <f>$M$48</f>
+        <v/>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>Rewards</t>
+        </is>
+      </c>
+      <c r="B59" s="8">
+        <f>0</f>
+        <v/>
+      </c>
+      <c r="C59" s="8">
+        <f>0</f>
+        <v/>
+      </c>
+      <c r="D59" s="8">
+        <f>MIN($B$7,$B$6*D51)</f>
+        <v/>
+      </c>
+      <c r="E59" s="8">
+        <f>MIN($B$7,$B$6*E51)</f>
+        <v/>
+      </c>
+      <c r="F59" s="8">
+        <f>MIN($B$7,$B$6*F51)</f>
+        <v/>
+      </c>
+      <c r="G59" s="8">
+        <f>MIN($B$7,$B$6*G51)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="2" t="inlineStr">
+        <is>
+          <t>Costs</t>
+        </is>
+      </c>
+      <c r="B60" s="8">
+        <f>SUM(B53:B59)</f>
+        <v/>
+      </c>
+      <c r="C60" s="8">
+        <f>SUM(C53:C59)</f>
+        <v/>
+      </c>
+      <c r="D60" s="8">
+        <f>SUM(D53:D59)</f>
+        <v/>
+      </c>
+      <c r="E60" s="8">
+        <f>SUM(E53:E59)</f>
+        <v/>
+      </c>
+      <c r="F60" s="8">
+        <f>SUM(F53:F59)</f>
+        <v/>
+      </c>
+      <c r="G60" s="8">
+        <f>SUM(G53:G59)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="2" t="inlineStr">
+        <is>
+          <t>Profit / loss</t>
+        </is>
+      </c>
+      <c r="B61" s="8">
+        <f>B52-B60</f>
+        <v/>
+      </c>
+      <c r="C61" s="8">
+        <f>C52-C60</f>
+        <v/>
+      </c>
+      <c r="D61" s="8">
+        <f>D52-D60</f>
+        <v/>
+      </c>
+      <c r="E61" s="8">
+        <f>E52-E60</f>
+        <v/>
+      </c>
+      <c r="F61" s="8">
+        <f>F52-F60</f>
+        <v/>
+      </c>
+      <c r="G61" s="8">
+        <f>G52-G60</f>
+        <v/>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>P/L without AI tokens</t>
+        </is>
+      </c>
+      <c r="B62" s="8">
+        <f>B61+B54</f>
+        <v/>
+      </c>
+      <c r="C62" s="8">
+        <f>C61+C54</f>
+        <v/>
+      </c>
+      <c r="D62" s="8">
+        <f>D61+D54</f>
+        <v/>
+      </c>
+      <c r="E62" s="8">
+        <f>E61+E54</f>
+        <v/>
+      </c>
+      <c r="F62" s="8">
+        <f>F61+F54</f>
+        <v/>
+      </c>
+      <c r="G62" s="8">
+        <f>G61+G54</f>
+        <v/>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>Cumulative P/L</t>
+        </is>
+      </c>
+      <c r="B63" s="8">
+        <f>B61</f>
+        <v/>
+      </c>
+      <c r="C63" s="8">
+        <f>B63+C61</f>
+        <v/>
+      </c>
+      <c r="D63" s="8">
+        <f>C63+D61</f>
+        <v/>
+      </c>
+      <c r="E63" s="8">
+        <f>D63+E61</f>
+        <v/>
+      </c>
+      <c r="F63" s="8">
+        <f>E63+F61</f>
+        <v/>
+      </c>
+      <c r="G63" s="8">
+        <f>F63+G61</f>
+        <v/>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="2" t="inlineStr">
+        <is>
+          <t>Break-even month</t>
+        </is>
+      </c>
+      <c r="B64">
+        <f>IFERROR(INDEX($B$49:$G$49,MATCH(TRUE,INDEX($B$61:$G$61&gt;=0,0),0)),"Not in 6 months")</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -690,14 +2807,13 @@
         <f>SUM(B2:B9)</f>
         <v/>
       </c>
-      <c r="C10" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3774,7 +5890,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -6842,7 +8958,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -9907,7 +12023,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -10273,7 +12389,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
Finance Budget v3: founder's real numbers, ₹10k/month lean plan, lean P&L, caps cut
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0191SJ1qAdm8xL7m212nsCqQ
</commit_message>
<xml_diff>
--- a/docs/finance/hostelzy-money.xlsx
+++ b/docs/finance/hostelzy-money.xlsx
@@ -456,7 +456,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B9"/>
+  <dimension ref="A1:B10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -552,6 +552,16 @@
       <c r="B9" t="inlineStr">
         <is>
           <t>Bills tab: every account the app needs, cost and due date. P&amp;L tab: 6-month P&amp;L at 20/50/100 hostels; edit yellow cells.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Budget v3 (2026-10-04): ₹10,000 a month to Hostelzy. Budget and P&amp;L tabs use the lean numbers.</t>
         </is>
       </c>
     </row>
@@ -1029,7 +1039,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>Assumptions (edit the yellow cells)</t>
+          <t>Assumptions (edit the yellow cells) · Budget v3 lean plan, 2026-10-04</t>
         </is>
       </c>
     </row>
@@ -1090,7 +1100,7 @@
         </is>
       </c>
       <c r="B7" s="6" t="n">
-        <v>5000</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="8">
@@ -1100,7 +1110,7 @@
         </is>
       </c>
       <c r="B8" s="6" t="n">
-        <v>10000</v>
+        <v>2300</v>
       </c>
     </row>
     <row r="9">
@@ -1110,19 +1120,20 @@
         </is>
       </c>
       <c r="B9" s="6" t="n">
-        <v>4260</v>
+        <v>2400</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Tech base from month 2 (₹, + SMS)</t>
+          <t>Supabase Pro from 10 paying hostels (₹)</t>
         </is>
       </c>
       <c r="B10" s="6" t="n">
-        <v>3360</v>
-      </c>
-    </row>
+        <v>2900</v>
+      </c>
+    </row>
+    <row r="11"/>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
@@ -1135,7 +1146,7 @@
         </is>
       </c>
       <c r="I12" s="6" t="n">
-        <v>500</v>
+        <v>0</v>
       </c>
       <c r="J12" t="inlineStr">
         <is>
@@ -1151,7 +1162,7 @@
         </is>
       </c>
       <c r="M12" s="6" t="n">
-        <v>1000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="13">
@@ -1288,23 +1299,23 @@
         <v/>
       </c>
       <c r="C17" s="8">
-        <f>$B$10+$I$12</f>
+        <f>IF(C15&gt;=10,$B$10,0)+$I$12</f>
         <v/>
       </c>
       <c r="D17" s="8">
-        <f>$B$10+$I$12</f>
+        <f>IF(D15&gt;=10,$B$10,0)+$I$12</f>
         <v/>
       </c>
       <c r="E17" s="8">
-        <f>$B$10+$I$12</f>
+        <f>IF(E15&gt;=10,$B$10,0)+$I$12</f>
         <v/>
       </c>
       <c r="F17" s="8">
-        <f>$B$10+$I$12</f>
+        <f>IF(F15&gt;=10,$B$10,0)+$I$12</f>
         <v/>
       </c>
       <c r="G17" s="8">
-        <f>$B$10+$I$12</f>
+        <f>IF(G15&gt;=10,$B$10,0)+$I$12</f>
         <v/>
       </c>
     </row>
@@ -1408,27 +1419,27 @@
         </is>
       </c>
       <c r="B21" s="8">
-        <f>3000</f>
+        <f>2000</f>
         <v/>
       </c>
       <c r="C21" s="8">
-        <f>IF(C14&gt;B14,3000,1000)</f>
+        <f>IF(C14&gt;B14,2000,1000)</f>
         <v/>
       </c>
       <c r="D21" s="8">
-        <f>IF(D14&gt;C14,3000,1000)</f>
+        <f>IF(D14&gt;C14,2000,1000)</f>
         <v/>
       </c>
       <c r="E21" s="8">
-        <f>IF(E14&gt;D14,3000,1000)</f>
+        <f>IF(E14&gt;D14,2000,1000)</f>
         <v/>
       </c>
       <c r="F21" s="8">
-        <f>IF(F14&gt;E14,3000,1000)</f>
+        <f>IF(F14&gt;E14,2000,1000)</f>
         <v/>
       </c>
       <c r="G21" s="8">
-        <f>IF(G14&gt;F14,3000,1000)</f>
+        <f>IF(G14&gt;F14,2000,1000)</f>
         <v/>
       </c>
     </row>
@@ -1629,6 +1640,7 @@
         <v/>
       </c>
     </row>
+    <row r="29"/>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
@@ -1641,23 +1653,23 @@
         </is>
       </c>
       <c r="I30" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>Hold pay ₹/mo</t>
+        </is>
+      </c>
+      <c r="K30" s="6" t="n">
         <v>1000</v>
       </c>
-      <c r="J30" t="inlineStr">
-        <is>
-          <t>Hold pay ₹/mo</t>
-        </is>
-      </c>
-      <c r="K30" s="6" t="n">
-        <v>2000</v>
-      </c>
       <c r="L30" t="inlineStr">
         <is>
           <t>Ads ₹/mo</t>
         </is>
       </c>
       <c r="M30" s="6" t="n">
-        <v>2000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="31">
@@ -1794,23 +1806,23 @@
         <v/>
       </c>
       <c r="C35" s="8">
-        <f>$B$10+$I$30</f>
+        <f>IF(C33&gt;=10,$B$10,0)+$I$30</f>
         <v/>
       </c>
       <c r="D35" s="8">
-        <f>$B$10+$I$30</f>
+        <f>IF(D33&gt;=10,$B$10,0)+$I$30</f>
         <v/>
       </c>
       <c r="E35" s="8">
-        <f>$B$10+$I$30</f>
+        <f>IF(E33&gt;=10,$B$10,0)+$I$30</f>
         <v/>
       </c>
       <c r="F35" s="8">
-        <f>$B$10+$I$30</f>
+        <f>IF(F33&gt;=10,$B$10,0)+$I$30</f>
         <v/>
       </c>
       <c r="G35" s="8">
-        <f>$B$10+$I$30</f>
+        <f>IF(G33&gt;=10,$B$10,0)+$I$30</f>
         <v/>
       </c>
     </row>
@@ -1914,27 +1926,27 @@
         </is>
       </c>
       <c r="B39" s="8">
-        <f>3000</f>
+        <f>2000</f>
         <v/>
       </c>
       <c r="C39" s="8">
-        <f>IF(C32&gt;B32,3000,1000)</f>
+        <f>IF(C32&gt;B32,2000,1000)</f>
         <v/>
       </c>
       <c r="D39" s="8">
-        <f>IF(D32&gt;C32,3000,1000)</f>
+        <f>IF(D32&gt;C32,2000,1000)</f>
         <v/>
       </c>
       <c r="E39" s="8">
-        <f>IF(E32&gt;D32,3000,1000)</f>
+        <f>IF(E32&gt;D32,2000,1000)</f>
         <v/>
       </c>
       <c r="F39" s="8">
-        <f>IF(F32&gt;E32,3000,1000)</f>
+        <f>IF(F32&gt;E32,2000,1000)</f>
         <v/>
       </c>
       <c r="G39" s="8">
-        <f>IF(G32&gt;F32,3000,1000)</f>
+        <f>IF(G32&gt;F32,2000,1000)</f>
         <v/>
       </c>
     </row>
@@ -2135,6 +2147,7 @@
         <v/>
       </c>
     </row>
+    <row r="47"/>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
@@ -2147,7 +2160,7 @@
         </is>
       </c>
       <c r="I48" s="6" t="n">
-        <v>2000</v>
+        <v>0</v>
       </c>
       <c r="J48" t="inlineStr">
         <is>
@@ -2155,7 +2168,7 @@
         </is>
       </c>
       <c r="K48" s="6" t="n">
-        <v>4000</v>
+        <v>1000</v>
       </c>
       <c r="L48" t="inlineStr">
         <is>
@@ -2163,7 +2176,7 @@
         </is>
       </c>
       <c r="M48" s="6" t="n">
-        <v>2000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="49">
@@ -2300,23 +2313,23 @@
         <v/>
       </c>
       <c r="C53" s="8">
-        <f>$B$10+$I$48</f>
+        <f>IF(C51&gt;=10,$B$10,0)+$I$48</f>
         <v/>
       </c>
       <c r="D53" s="8">
-        <f>$B$10+$I$48</f>
+        <f>IF(D51&gt;=10,$B$10,0)+$I$48</f>
         <v/>
       </c>
       <c r="E53" s="8">
-        <f>$B$10+$I$48</f>
+        <f>IF(E51&gt;=10,$B$10,0)+$I$48</f>
         <v/>
       </c>
       <c r="F53" s="8">
-        <f>$B$10+$I$48</f>
+        <f>IF(F51&gt;=10,$B$10,0)+$I$48</f>
         <v/>
       </c>
       <c r="G53" s="8">
-        <f>$B$10+$I$48</f>
+        <f>IF(G51&gt;=10,$B$10,0)+$I$48</f>
         <v/>
       </c>
     </row>
@@ -2420,27 +2433,27 @@
         </is>
       </c>
       <c r="B57" s="8">
-        <f>3000</f>
+        <f>2000</f>
         <v/>
       </c>
       <c r="C57" s="8">
-        <f>IF(C50&gt;B50,3000,1000)</f>
+        <f>IF(C50&gt;B50,2000,1000)</f>
         <v/>
       </c>
       <c r="D57" s="8">
-        <f>IF(D50&gt;C50,3000,1000)</f>
+        <f>IF(D50&gt;C50,2000,1000)</f>
         <v/>
       </c>
       <c r="E57" s="8">
-        <f>IF(E50&gt;D50,3000,1000)</f>
+        <f>IF(E50&gt;D50,2000,1000)</f>
         <v/>
       </c>
       <c r="F57" s="8">
-        <f>IF(F50&gt;E50,3000,1000)</f>
+        <f>IF(F50&gt;E50,2000,1000)</f>
         <v/>
       </c>
       <c r="G57" s="8">
-        <f>IF(G50&gt;F50,3000,1000)</f>
+        <f>IF(G50&gt;F50,2000,1000)</f>
         <v/>
       </c>
     </row>
@@ -2663,7 +2676,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Bucket</t>
+          <t>Bucket (Budget v3: ₹10,000 a month, 2026-10-04)</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
@@ -2684,11 +2697,11 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>5000</v>
+        <v>0</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Supabase, Play, maps, domain</t>
+          <t>₹0 now. Play ₹2,400 once (from buffer). Supabase Pro ₹2,900 only from 10 paying hostels, paid from revenue</t>
         </is>
       </c>
     </row>
@@ -2699,11 +2712,11 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>10000</v>
+        <v>2300</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Claude plan; fill real bill</t>
+          <t>Pro-level Claude plan; fill your real bill</t>
         </is>
       </c>
     </row>
@@ -2714,11 +2727,11 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>5000</v>
+        <v>1000</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>PROPOSED cap, plan.md §6</t>
+          <t>Cash referrals only; next-stay credits are invoice credits</t>
         </is>
       </c>
     </row>
@@ -2729,11 +2742,11 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>8000</v>
+        <v>1000</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Partners / ambassadors</t>
+          <t>Hold pay for all partners. ₹200/paying owner is paid from that owner's payment</t>
         </is>
       </c>
     </row>
@@ -2744,11 +2757,11 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>4000</v>
+        <v>1500</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>QR posters, stickers</t>
+          <t>~10 hostels × ₹150</t>
         </is>
       </c>
     </row>
@@ -2759,7 +2772,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>3000</v>
+        <v>2000</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -2774,11 +2787,11 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>2000</v>
+        <v>0</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Instagram boosts, test only</t>
+          <t>Free reels only</t>
         </is>
       </c>
     </row>
@@ -2789,11 +2802,11 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>3000</v>
+        <v>2200</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Plus anything unused</t>
+          <t>Buffer: pays Play in Oct, then rolls over</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Finance: Claude free, founder pays Play + Supabase Pro now; where-to-pay table, P&L updated
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0191SJ1qAdm8xL7m212nsCqQ
</commit_message>
<xml_diff>
--- a/docs/finance/hostelzy-money.xlsx
+++ b/docs/finance/hostelzy-money.xlsx
@@ -677,7 +677,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>1 Nov 2026</t>
+          <t>Now (before real owners' data)</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -769,14 +769,14 @@
         </is>
       </c>
       <c r="C6" s="4" t="n">
-        <v>1000</v>
+        <v>0</v>
       </c>
       <c r="D6" s="4" t="n">
         <v>0</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Nov 2026 (card)</t>
+          <t>Later, optional</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -897,11 +897,11 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>$4/mo when repo private</t>
+          <t>Later: $4/mo only if repo goes private</t>
         </is>
       </c>
       <c r="C10" s="4" t="n">
-        <v>460</v>
+        <v>0</v>
       </c>
       <c r="D10" s="4" t="n">
         <v>0</v>
@@ -930,11 +930,11 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Your plan</t>
+          <t>Free for the founder</t>
         </is>
       </c>
       <c r="C11" s="4" t="n">
-        <v>10000</v>
+        <v>0</v>
       </c>
       <c r="D11" s="4" t="n">
         <v>0</v>
@@ -1110,23 +1110,23 @@
         </is>
       </c>
       <c r="B8" s="6" t="n">
-        <v>2300</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Tech month 1 (₹)</t>
+          <t>Tech month 1 (₹, Play once + Supabase Pro)</t>
         </is>
       </c>
       <c r="B9" s="6" t="n">
-        <v>2400</v>
+        <v>5300</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Supabase Pro from 10 paying hostels (₹)</t>
+          <t>Supabase Pro per month (₹)</t>
         </is>
       </c>
       <c r="B10" s="6" t="n">
@@ -1299,23 +1299,23 @@
         <v/>
       </c>
       <c r="C17" s="8">
-        <f>IF(C15&gt;=10,$B$10,0)+$I$12</f>
+        <f>$B$10+$I$12</f>
         <v/>
       </c>
       <c r="D17" s="8">
-        <f>IF(D15&gt;=10,$B$10,0)+$I$12</f>
+        <f>$B$10+$I$12</f>
         <v/>
       </c>
       <c r="E17" s="8">
-        <f>IF(E15&gt;=10,$B$10,0)+$I$12</f>
+        <f>$B$10+$I$12</f>
         <v/>
       </c>
       <c r="F17" s="8">
-        <f>IF(F15&gt;=10,$B$10,0)+$I$12</f>
+        <f>$B$10+$I$12</f>
         <v/>
       </c>
       <c r="G17" s="8">
-        <f>IF(G15&gt;=10,$B$10,0)+$I$12</f>
+        <f>$B$10+$I$12</f>
         <v/>
       </c>
     </row>
@@ -1806,23 +1806,23 @@
         <v/>
       </c>
       <c r="C35" s="8">
-        <f>IF(C33&gt;=10,$B$10,0)+$I$30</f>
+        <f>$B$10+$I$30</f>
         <v/>
       </c>
       <c r="D35" s="8">
-        <f>IF(D33&gt;=10,$B$10,0)+$I$30</f>
+        <f>$B$10+$I$30</f>
         <v/>
       </c>
       <c r="E35" s="8">
-        <f>IF(E33&gt;=10,$B$10,0)+$I$30</f>
+        <f>$B$10+$I$30</f>
         <v/>
       </c>
       <c r="F35" s="8">
-        <f>IF(F33&gt;=10,$B$10,0)+$I$30</f>
+        <f>$B$10+$I$30</f>
         <v/>
       </c>
       <c r="G35" s="8">
-        <f>IF(G33&gt;=10,$B$10,0)+$I$30</f>
+        <f>$B$10+$I$30</f>
         <v/>
       </c>
     </row>
@@ -2313,23 +2313,23 @@
         <v/>
       </c>
       <c r="C53" s="8">
-        <f>IF(C51&gt;=10,$B$10,0)+$I$48</f>
+        <f>$B$10+$I$48</f>
         <v/>
       </c>
       <c r="D53" s="8">
-        <f>IF(D51&gt;=10,$B$10,0)+$I$48</f>
+        <f>$B$10+$I$48</f>
         <v/>
       </c>
       <c r="E53" s="8">
-        <f>IF(E51&gt;=10,$B$10,0)+$I$48</f>
+        <f>$B$10+$I$48</f>
         <v/>
       </c>
       <c r="F53" s="8">
-        <f>IF(F51&gt;=10,$B$10,0)+$I$48</f>
+        <f>$B$10+$I$48</f>
         <v/>
       </c>
       <c r="G53" s="8">
-        <f>IF(G51&gt;=10,$B$10,0)+$I$48</f>
+        <f>$B$10+$I$48</f>
         <v/>
       </c>
     </row>
@@ -2697,11 +2697,11 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0</v>
+        <v>2900</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>₹0 now. Play ₹2,400 once (from buffer). Supabase Pro ₹2,900 only from 10 paying hostels, paid from revenue</t>
+          <t>Supabase Pro from now. Play ₹2,400 once in Oct (from buffer)</t>
         </is>
       </c>
     </row>
@@ -2712,11 +2712,11 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>2300</v>
+        <v>0</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Pro-level Claude plan; fill your real bill</t>
+          <t>Claude is free for the founder (2026-10-04)</t>
         </is>
       </c>
     </row>
@@ -2802,7 +2802,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>2200</v>
+        <v>1600</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>

</xml_diff>